<commit_message>
feat: Nuevo modulo, gestion de horas para colaboradores
</commit_message>
<xml_diff>
--- a/proyectos_diseno/BASES_DE_DATOS/Disenadores.xlsx
+++ b/proyectos_diseno/BASES_DE_DATOS/Disenadores.xlsx
@@ -10,7 +10,7 @@
     <sheet name="DISENADORES" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DISENADORES'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DISENADORES'!$A$1:$K$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -147,9 +147,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TB_DISENADORES" displayName="TB_DISENADORES" ref="A1:I9" headerRowCount="1">
-  <autoFilter ref="A1:I9"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TB_DISENADORES" displayName="TB_DISENADORES" ref="A1:K10" headerRowCount="1">
+  <autoFilter ref="A1:K10"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="nombre"/>
     <tableColumn id="3" name="color"/>
@@ -159,6 +159,8 @@
     <tableColumn id="7" name="almuerzo_inicio"/>
     <tableColumn id="8" name="almuerzo_fin"/>
     <tableColumn id="9" name="activo"/>
+    <tableColumn id="10" name="descansos"/>
+    <tableColumn id="11" name="dias_laborales"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -453,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -465,6 +467,8 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -513,6 +517,16 @@
           <t>activo</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>descansos</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dias_laborales</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -556,6 +570,16 @@
       <c r="I2" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>[["12:00", "13:00"]]</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -599,6 +623,8 @@
       <c r="I3" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -642,6 +668,8 @@
       <c r="I4" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -685,6 +713,8 @@
       <c r="I5" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -728,6 +758,8 @@
       <c r="I6" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -771,6 +803,8 @@
       <c r="I7" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -814,6 +848,8 @@
       <c r="I8" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -857,9 +893,64 @@
       <c r="I9" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>369a1665-edbd-4bc2-b94c-54b9845f665e</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Prueba#1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>#ff0a0a</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>[["12:25", "13:00"]]</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:K10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
refactor: act usuario // rol
</commit_message>
<xml_diff>
--- a/proyectos_diseno/BASES_DE_DATOS/Disenadores.xlsx
+++ b/proyectos_diseno/BASES_DE_DATOS/Disenadores.xlsx
@@ -623,8 +623,16 @@
       <c r="I3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>[["12:00", "13:00"]]</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">

</xml_diff>